<commit_message>
Created gps name to planting name lookup.
</commit_message>
<xml_diff>
--- a/output_tables/p_gps_pts_Jn_mult.xlsx
+++ b/output_tables/p_gps_pts_Jn_mult.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofwa-my.sharepoint.com/personal/peter_dowty_dnr_wa_gov/Documents/projects/seagrass_restoration_data_2026/output_tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FECCA289-D33D-4F12-9A36-21C62E2CAB59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="8_{FECCA289-D33D-4F12-9A36-21C62E2CAB59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA273A31-6907-4D4B-9CBC-4BC1161B1E88}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="30" windowWidth="28800" windowHeight="15360" xr2:uid="{010213C7-2629-45B6-81B0-C8532EDDC33D}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="131">
   <si>
     <t>site_name</t>
   </si>
@@ -1300,6 +1300,9 @@
       <c r="D1" t="s">
         <v>2</v>
       </c>
+      <c r="E1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
@@ -1331,6 +1334,9 @@
       <c r="D3" t="s">
         <v>5</v>
       </c>
+      <c r="E3" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
@@ -1362,6 +1368,9 @@
       <c r="D5" t="s">
         <v>5</v>
       </c>
+      <c r="E5" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
@@ -1393,6 +1402,9 @@
       <c r="D7" t="s">
         <v>5</v>
       </c>
+      <c r="E7" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
@@ -1424,6 +1436,9 @@
       <c r="D9" t="s">
         <v>5</v>
       </c>
+      <c r="E9" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
@@ -1455,6 +1470,9 @@
       <c r="D11" t="s">
         <v>5</v>
       </c>
+      <c r="E11" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
@@ -1486,6 +1504,9 @@
       <c r="D13" t="s">
         <v>5</v>
       </c>
+      <c r="E13" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
@@ -1500,6 +1521,9 @@
       <c r="D14" t="s">
         <v>5</v>
       </c>
+      <c r="E14" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
@@ -1514,6 +1538,9 @@
       <c r="D15" t="s">
         <v>5</v>
       </c>
+      <c r="E15" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
@@ -1545,6 +1572,9 @@
       <c r="D17" t="s">
         <v>5</v>
       </c>
+      <c r="E17" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
@@ -1576,6 +1606,9 @@
       <c r="D19" t="s">
         <v>5</v>
       </c>
+      <c r="E19" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
@@ -1607,6 +1640,9 @@
       <c r="D21" t="s">
         <v>5</v>
       </c>
+      <c r="E21" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
@@ -1638,6 +1674,9 @@
       <c r="D23" t="s">
         <v>5</v>
       </c>
+      <c r="E23" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
@@ -1669,6 +1708,9 @@
       <c r="D25" t="s">
         <v>5</v>
       </c>
+      <c r="E25" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
@@ -1683,6 +1725,9 @@
       <c r="D26" t="s">
         <v>5</v>
       </c>
+      <c r="E26" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
@@ -1697,6 +1742,9 @@
       <c r="D27" t="s">
         <v>5</v>
       </c>
+      <c r="E27" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28">
@@ -1728,6 +1776,9 @@
       <c r="D29" t="s">
         <v>5</v>
       </c>
+      <c r="E29" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30">
@@ -1742,6 +1793,9 @@
       <c r="D30" t="s">
         <v>5</v>
       </c>
+      <c r="E30" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31">
@@ -1756,6 +1810,9 @@
       <c r="D31" t="s">
         <v>5</v>
       </c>
+      <c r="E31" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32">
@@ -1787,6 +1844,9 @@
       <c r="D33" t="s">
         <v>5</v>
       </c>
+      <c r="E33" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34">
@@ -1801,6 +1861,9 @@
       <c r="D34" t="s">
         <v>5</v>
       </c>
+      <c r="E34" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35">
@@ -1815,6 +1878,9 @@
       <c r="D35" t="s">
         <v>5</v>
       </c>
+      <c r="E35" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36">
@@ -1846,6 +1912,9 @@
       <c r="D37" t="s">
         <v>5</v>
       </c>
+      <c r="E37" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38">
@@ -1877,6 +1946,9 @@
       <c r="D39" t="s">
         <v>5</v>
       </c>
+      <c r="E39" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
@@ -1908,6 +1980,9 @@
       <c r="D41" t="s">
         <v>5</v>
       </c>
+      <c r="E41" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42">
@@ -1922,6 +1997,9 @@
       <c r="D42" t="s">
         <v>5</v>
       </c>
+      <c r="E42" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43">
@@ -1936,6 +2014,9 @@
       <c r="D43" t="s">
         <v>5</v>
       </c>
+      <c r="E43" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44">
@@ -1967,6 +2048,9 @@
       <c r="D45" t="s">
         <v>5</v>
       </c>
+      <c r="E45" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46">
@@ -1981,6 +2065,9 @@
       <c r="D46" t="s">
         <v>5</v>
       </c>
+      <c r="E46" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47">
@@ -1995,6 +2082,9 @@
       <c r="D47" t="s">
         <v>5</v>
       </c>
+      <c r="E47" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48">
@@ -2026,6 +2116,9 @@
       <c r="D49" t="s">
         <v>5</v>
       </c>
+      <c r="E49" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50">
@@ -2040,6 +2133,9 @@
       <c r="D50" t="s">
         <v>5</v>
       </c>
+      <c r="E50" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51">
@@ -2054,6 +2150,9 @@
       <c r="D51" t="s">
         <v>5</v>
       </c>
+      <c r="E51" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52">
@@ -2085,6 +2184,9 @@
       <c r="D53" t="s">
         <v>5</v>
       </c>
+      <c r="E53" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54">
@@ -2116,6 +2218,9 @@
       <c r="D55" t="s">
         <v>5</v>
       </c>
+      <c r="E55" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56">
@@ -2147,6 +2252,9 @@
       <c r="D57" t="s">
         <v>5</v>
       </c>
+      <c r="E57" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58">
@@ -2161,6 +2269,9 @@
       <c r="D58" t="s">
         <v>5</v>
       </c>
+      <c r="E58" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59">
@@ -2175,6 +2286,9 @@
       <c r="D59" t="s">
         <v>5</v>
       </c>
+      <c r="E59" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60">
@@ -2206,6 +2320,9 @@
       <c r="D61" t="s">
         <v>5</v>
       </c>
+      <c r="E61" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62">
@@ -2220,6 +2337,9 @@
       <c r="D62" t="s">
         <v>5</v>
       </c>
+      <c r="E62" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63">
@@ -2234,6 +2354,9 @@
       <c r="D63" t="s">
         <v>5</v>
       </c>
+      <c r="E63" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64">
@@ -2265,6 +2388,9 @@
       <c r="D65" t="s">
         <v>5</v>
       </c>
+      <c r="E65" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66">
@@ -2279,6 +2405,9 @@
       <c r="D66" t="s">
         <v>5</v>
       </c>
+      <c r="E66" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67">
@@ -2293,6 +2422,9 @@
       <c r="D67" t="s">
         <v>5</v>
       </c>
+      <c r="E67" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68">
@@ -2324,6 +2456,9 @@
       <c r="D69" t="s">
         <v>5</v>
       </c>
+      <c r="E69" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70">
@@ -2338,6 +2473,9 @@
       <c r="D70" t="s">
         <v>5</v>
       </c>
+      <c r="E70" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71">
@@ -2352,6 +2490,9 @@
       <c r="D71" t="s">
         <v>5</v>
       </c>
+      <c r="E71" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72">
@@ -2383,6 +2524,9 @@
       <c r="D73" t="s">
         <v>5</v>
       </c>
+      <c r="E73" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74">
@@ -2414,6 +2558,9 @@
       <c r="D75" t="s">
         <v>5</v>
       </c>
+      <c r="E75" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76">
@@ -2428,6 +2575,9 @@
       <c r="D76" t="s">
         <v>5</v>
       </c>
+      <c r="E76" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77">
@@ -2441,6 +2591,9 @@
       </c>
       <c r="D77" t="s">
         <v>5</v>
+      </c>
+      <c r="E77" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>